<commit_message>
Small fixes and styling changes
</commit_message>
<xml_diff>
--- a/documentation/csvTemplate.xlsx
+++ b/documentation/csvTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timco\Desktop\SoftwareProject\gosmartlib\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D70A327-6055-499B-836E-F8A26F10CBBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59D58D3A-D8DF-4865-AE18-740AAF6F7EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6870" yWindow="1335" windowWidth="26070" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1650" yWindow="2205" windowWidth="26070" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Titel</t>
   </si>
@@ -34,12 +34,6 @@
   </si>
   <si>
     <t>ISBN</t>
-  </si>
-  <si>
-    <t>Taal</t>
-  </si>
-  <si>
-    <t>Beschrijving</t>
   </si>
   <si>
     <t>Conditie_nieuw</t>
@@ -87,7 +81,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -122,19 +116,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -164,15 +145,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -453,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="2"/>
@@ -464,11 +444,9 @@
     <col min="7" max="7" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.5703125" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -479,40 +457,29 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1:J1048576" xr:uid="{BD54D82C-BCD2-4A99-B11D-CAB70F64C0C1}">
-      <formula1>"NEDERLANDS,FRANS,ENGELS,DUITS,ANDERE"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>